<commit_message>
Weave in certification/bloodline/price/colors info (values cards + FAQ)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1848,7 +1848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1924,6 +1924,30 @@
       <c r="B6" s="2" t="inlineStr">
         <is>
           <t>欢迎通过页面下方的微信或电话直接咨询我们。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>小猫的价格范围？</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>5000–30000 元不等，具体取决于脸版品相、骨量结构与毛量毛色，欢迎微信咨询心仪的小猫。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>猫舍有哪些花色？</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>银虎斑、棕虎斑、烟灰系、凯米尔、红虎斑、纯白、纯黑、蓝虎斑等。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FAQ: move 还有其他问题 to last position
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1918,36 +1918,36 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>还有其他问题？</t>
+          <t>小猫的价格范围？</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>欢迎通过页面下方的微信或电话直接咨询我们。</t>
+          <t>5000–30000 元不等，具体取决于脸版品相、骨量结构与毛量毛色，欢迎微信咨询心仪的小猫。</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>小猫的价格范围？</t>
+          <t>猫舍有哪些花色？</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>5000–30000 元不等，具体取决于脸版品相、骨量结构与毛量毛色，欢迎微信咨询心仪的小猫。</t>
+          <t>银虎斑、棕虎斑、烟灰系、凯米尔、红虎斑、纯白、纯黑、蓝虎斑等。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>猫舍有哪些花色？</t>
+          <t>还有其他问题？</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>银虎斑、棕虎斑、烟灰系、凯米尔、红虎斑、纯白、纯黑、蓝虎斑等。</t>
+          <t>欢迎通过页面下方的微信或电话直接咨询我们。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record Aug 2 sales (silver tabby boy -> Heilongjiang, smoke boy -> Chongqing); fix stray image path
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -607,7 +607,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -615,7 +615,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>重庆</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -719,7 +723,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -727,7 +731,11 @@
           <t>2026-06-05</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>黑龙江</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1591,7 +1599,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>assets/1785912551260-jplefm937nk.jpeg, assets/videos/02.mp4</t>
+          <t>assets/1785912551260-jplefm937nk.jpeg</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1731,7 +1739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1770,6 +1778,40 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Shakoshako 猫舍官网全新上线，欢迎关注！</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>出售</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>银虎斑弟弟找到新家，前往黑龙江。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>出售</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>烟灰色弟弟找到新家，前往重庆。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Zouzou diary: real birthday 2-20, family-found 7-02, carrier photo on departure page; optional J/K milestone columns
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -504,6 +504,16 @@
           <t>名字</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>定新家日期</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>出发照片</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1152,7 +1162,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2026-02-20</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1173,6 +1183,16 @@
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>驺驺</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>assets/diary/zouzou-depart.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Diary milestones: vaccine, serology, dated departure (future shows as planned) — Zouzou 7-02/8-03/11-03
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K43"/>
+  <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -514,6 +514,21 @@
           <t>出发照片</t>
         </is>
       </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>打疫苗日期</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>血清检测日期</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>出发日期</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1193,6 +1208,21 @@
       <c r="K24" t="inlineStr">
         <is>
           <t>assets/diary/zouzou-depart.jpg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-11-03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Zouzou: hide departure date for now; non-date departure text counts as planned
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1220,11 +1220,6 @@
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>2026-11-03</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Zouzou feedback: dated last Thursday, five months ten days old
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1905,7 +1905,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1915,7 +1915,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>在荷兰的新家适应得很好，活泼又粘人。</t>
+          <t>五个月10天了。</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Excel-free fast path: Action converts xlsx to sheets.json, site parses JSON directly (xlsx lib only as fallback); weight records diary page — Zouzou 6.2 jin
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -444,7 +444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:O43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -529,6 +529,11 @@
           <t>出发日期</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>体重记录</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1218,6 +1223,11 @@
       <c r="M24" t="inlineStr">
         <is>
           <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2026-07-30 · 6.2斤</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop mismatched photo from 7-30 feedback (pending correct one)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1928,11 +1928,7 @@
           <t>五个月10天了。</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>assets/feedback/zouzou-1.jpg</t>
-        </is>
-      </c>
+      <c r="D2" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Diary pages sort chronologically; feedback entries slot by date (7-30 before serology); restore feedback photo
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1928,7 +1928,11 @@
           <t>五个月10天了。</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>assets/feedback/zouzou-1.jpg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Diary: dates inline in page titles, image-less pages flat, growth records own photos (7-30 entry moved from feedback)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kittens.xlsx
+++ b/data/kittens.xlsx
@@ -1227,7 +1227,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-07-30 · 6.2斤</t>
+          <t>2026-07-30 · 6.2斤 · 五个月10天了 · assets/feedback/zouzou-1.jpg</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1909,28 +1909,6 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>图片路径</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-30</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>驺驺</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>五个月10天了。</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>assets/feedback/zouzou-1.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>